<commit_message>
payroll status added; updated site requirements
</commit_message>
<xml_diff>
--- a/public/SITE REQUIREMENT TAB.xlsx
+++ b/public/SITE REQUIREMENT TAB.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GRID WATCH ENHANCEMENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04071FBB-D9EA-4E0E-AFA1-947E0F3D14DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883D7C5D-CE34-4077-B305-ECD3E08C7213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E68F1FC1-89F5-4CA1-B04B-E36E50ABA536}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{E68F1FC1-89F5-4CA1-B04B-E36E50ABA536}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="SITE REQUIREMENT" sheetId="1" r:id="rId1"/>
+    <sheet name="DPR" sheetId="2" r:id="rId2"/>
+    <sheet name="CONSUMABLES" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="171">
   <si>
     <t>S.NO.</t>
   </si>
@@ -104,6 +106,456 @@
   </si>
   <si>
     <t>SUB DESCRIPTION</t>
+  </si>
+  <si>
+    <t>DESCRIPTION</t>
+  </si>
+  <si>
+    <t>REMARKS</t>
+  </si>
+  <si>
+    <t>QTY.</t>
+  </si>
+  <si>
+    <t>S. No.</t>
+  </si>
+  <si>
+    <t>Welding Rod</t>
+  </si>
+  <si>
+    <t>Machine Oil</t>
+  </si>
+  <si>
+    <t>Nut Bolt</t>
+  </si>
+  <si>
+    <t>M6 / M8 / M10 / M12 / M16</t>
+  </si>
+  <si>
+    <t>Bullet Fastener</t>
+  </si>
+  <si>
+    <t>M8 / M10 / M12</t>
+  </si>
+  <si>
+    <t>Anchor Fastener</t>
+  </si>
+  <si>
+    <t>M8 / M10 / M12 / M16</t>
+  </si>
+  <si>
+    <t>Paint</t>
+  </si>
+  <si>
+    <t>Primer</t>
+  </si>
+  <si>
+    <t>1 / 2 / 3 / 4 Inch</t>
+  </si>
+  <si>
+    <t>Consumable Item</t>
+  </si>
+  <si>
+    <t>Common Size / Specification</t>
+  </si>
+  <si>
+    <t>2.5 / 3.15 / 4.0 mm</t>
+  </si>
+  <si>
+    <t>Cutting Wheel</t>
+  </si>
+  <si>
+    <t>4 / 5 / 7 Inch</t>
+  </si>
+  <si>
+    <t>Grinding Wheel</t>
+  </si>
+  <si>
+    <t>1 / 5 / 20 Ltr</t>
+  </si>
+  <si>
+    <t>4 / 8 / 10 Kg</t>
+  </si>
+  <si>
+    <t>Paint Brush</t>
+  </si>
+  <si>
+    <t>Teflon Tape</t>
+  </si>
+  <si>
+    <t>12 / 19 / 25 mm</t>
+  </si>
+  <si>
+    <t>Thread Sealant</t>
+  </si>
+  <si>
+    <t>50 / 100 / 250 gm</t>
+  </si>
+  <si>
+    <t>PTFE Sealant</t>
+  </si>
+  <si>
+    <t>100 / 250 gm</t>
+  </si>
+  <si>
+    <t>GI Pipe Jointing Compound</t>
+  </si>
+  <si>
+    <t>1 / 5 Kg</t>
+  </si>
+  <si>
+    <t>Gasket</t>
+  </si>
+  <si>
+    <t>1/2" to 6"</t>
+  </si>
+  <si>
+    <t>Rubber Sheet</t>
+  </si>
+  <si>
+    <t>2 / 3 / 5 mm</t>
+  </si>
+  <si>
+    <t>GI/MS Pipe</t>
+  </si>
+  <si>
+    <t>As Required</t>
+  </si>
+  <si>
+    <t>Pipe Nipples</t>
+  </si>
+  <si>
+    <t>1/2" / 3/4" / 1" / 1½"</t>
+  </si>
+  <si>
+    <t>GI Fittings</t>
+  </si>
+  <si>
+    <t>1/2" to 4"</t>
+  </si>
+  <si>
+    <t>MS Flanges</t>
+  </si>
+  <si>
+    <t>U-Clamp / Pipe Clamp</t>
+  </si>
+  <si>
+    <t>25 / 32 / 40 / 50 / 65 / 80 mm</t>
+  </si>
+  <si>
+    <t>Clevis Hanger</t>
+  </si>
+  <si>
+    <t>Threaded Rod</t>
+  </si>
+  <si>
+    <t>6 / 8 / 10 / 12 mm</t>
+  </si>
+  <si>
+    <t>GI Channel / Strut</t>
+  </si>
+  <si>
+    <t>41 × 41 mm</t>
+  </si>
+  <si>
+    <t>PVC Insulation Tape</t>
+  </si>
+  <si>
+    <t>18 mm</t>
+  </si>
+  <si>
+    <t>Cable Ties</t>
+  </si>
+  <si>
+    <t>100 / 200 / 300 mm</t>
+  </si>
+  <si>
+    <t>Electrical Cable Lugs</t>
+  </si>
+  <si>
+    <t>Heat Shrink Sleeve</t>
+  </si>
+  <si>
+    <t>Silicone Sealant</t>
+  </si>
+  <si>
+    <t>280 / 300 ml</t>
+  </si>
+  <si>
+    <t>Fire-Rated Sealant</t>
+  </si>
+  <si>
+    <t>300 / 600 ml</t>
+  </si>
+  <si>
+    <t>Fire Stop Material</t>
+  </si>
+  <si>
+    <t>Cable Gland</t>
+  </si>
+  <si>
+    <t>Various Sizes</t>
+  </si>
+  <si>
+    <t>Identification Labels</t>
+  </si>
+  <si>
+    <t>Pipe Identification Tape</t>
+  </si>
+  <si>
+    <t>Red / White</t>
+  </si>
+  <si>
+    <t>Emery Paper</t>
+  </si>
+  <si>
+    <t>80 / 120 / 180 Grit</t>
+  </si>
+  <si>
+    <t>Wire Brush</t>
+  </si>
+  <si>
+    <t>1 / 2 / 3 Inch</t>
+  </si>
+  <si>
+    <t>Cotton Waste</t>
+  </si>
+  <si>
+    <t>Cleaning Solvent</t>
+  </si>
+  <si>
+    <t>1 / 5 Ltr</t>
+  </si>
+  <si>
+    <t>Anti-Rust Paint</t>
+  </si>
+  <si>
+    <t>1 / 4 / 10 Ltr</t>
+  </si>
+  <si>
+    <t>Red Oxide Primer</t>
+  </si>
+  <si>
+    <t>SIZE / SPECIFICATION</t>
+  </si>
+  <si>
+    <t>Installation Fire Alarm Cable</t>
+  </si>
+  <si>
+    <t>2C × 1.5 / 2.5 Sq.mm</t>
+  </si>
+  <si>
+    <t>Installation Speaker Wire</t>
+  </si>
+  <si>
+    <t>M.S. Pipe Installation</t>
+  </si>
+  <si>
+    <t>25 / 32 / 50 / 65 / 80 / 100 / 150 / 200 mm</t>
+  </si>
+  <si>
+    <t>G.I. Pipe Installation</t>
+  </si>
+  <si>
+    <t>Elbow Installation</t>
+  </si>
+  <si>
+    <t>Tee Installation</t>
+  </si>
+  <si>
+    <t>Reducer Installation</t>
+  </si>
+  <si>
+    <t>Flange Installation</t>
+  </si>
+  <si>
+    <t>Grooved Coupling Installation</t>
+  </si>
+  <si>
+    <t>Union Installation</t>
+  </si>
+  <si>
+    <t>Valve Installation</t>
+  </si>
+  <si>
+    <t>Butterfly Valve Installation</t>
+  </si>
+  <si>
+    <t>50 / 65 / 80 / 100 / 150 / 200 mm</t>
+  </si>
+  <si>
+    <t>NRV Installation</t>
+  </si>
+  <si>
+    <t>Y-Strainer Installation</t>
+  </si>
+  <si>
+    <t>Fire Hydrant Installation</t>
+  </si>
+  <si>
+    <t>As Per Approved Drawing</t>
+  </si>
+  <si>
+    <t>Hose Reel Installation</t>
+  </si>
+  <si>
+    <t>Landing Valve Installation</t>
+  </si>
+  <si>
+    <t>63 mm / 2½"</t>
+  </si>
+  <si>
+    <t>Fire Hose Installation</t>
+  </si>
+  <si>
+    <t>15 / 20 / 30 m</t>
+  </si>
+  <si>
+    <t>Fire Hose Cabinet Installation</t>
+  </si>
+  <si>
+    <t>Sprinkler Installation</t>
+  </si>
+  <si>
+    <t>15 / 20 mm</t>
+  </si>
+  <si>
+    <t>Sprinkler Flexible Drop Installation</t>
+  </si>
+  <si>
+    <t>Sprinkler Head Installation</t>
+  </si>
+  <si>
+    <t>Upright / Pendent / Sidewall</t>
+  </si>
+  <si>
+    <t>Pipe Support Installation</t>
+  </si>
+  <si>
+    <t>M8 / M10 / M12 Threaded Rod</t>
+  </si>
+  <si>
+    <t>Pipe Clamp Installation</t>
+  </si>
+  <si>
+    <t>25–200 mm</t>
+  </si>
+  <si>
+    <t>MS Channel Support Installation</t>
+  </si>
+  <si>
+    <t>41 × 41 / 50 × 50 mm</t>
+  </si>
+  <si>
+    <t>Fire Pump Installation</t>
+  </si>
+  <si>
+    <t>Jockey Pump Installation</t>
+  </si>
+  <si>
+    <t>Diesel Pump Installation</t>
+  </si>
+  <si>
+    <t>Fire Water Tank Connection</t>
+  </si>
+  <si>
+    <t>Pressure Gauge Installation</t>
+  </si>
+  <si>
+    <t>Flow Switch Installation</t>
+  </si>
+  <si>
+    <t>Pressure Switch Installation</t>
+  </si>
+  <si>
+    <t>Test &amp; Drain Assembly Installation</t>
+  </si>
+  <si>
+    <t>Fire Alarm Panel Installation</t>
+  </si>
+  <si>
+    <t>Addressable / Conventional</t>
+  </si>
+  <si>
+    <t>Smoke Detector Installation</t>
+  </si>
+  <si>
+    <t>Heat Detector Installation</t>
+  </si>
+  <si>
+    <t>Manual Call Point Installation</t>
+  </si>
+  <si>
+    <t>Hooter / Sounder Installation</t>
+  </si>
+  <si>
+    <t>Speaker Installation</t>
+  </si>
+  <si>
+    <t>3 / 6 / 10 W</t>
+  </si>
+  <si>
+    <t>Strobe / Sounder Strobe Installation</t>
+  </si>
+  <si>
+    <t>Monitor Module Installation</t>
+  </si>
+  <si>
+    <t>Control Module Installation</t>
+  </si>
+  <si>
+    <t>Fire Alarm Junction Box Installation</t>
+  </si>
+  <si>
+    <t>Fire Alarm Cable Termination</t>
+  </si>
+  <si>
+    <t>Fire Alarm Cable Testing</t>
+  </si>
+  <si>
+    <t>Continuity / Insulation</t>
+  </si>
+  <si>
+    <t>Fire Fighting Pipe Welding</t>
+  </si>
+  <si>
+    <t>Pipe Threading / Grooving</t>
+  </si>
+  <si>
+    <t>Pipe Flushing</t>
+  </si>
+  <si>
+    <t>Hydrostatic Pressure Testing</t>
+  </si>
+  <si>
+    <t>As Per Specification</t>
+  </si>
+  <si>
+    <t>Fire Fighting System Testing</t>
+  </si>
+  <si>
+    <t>As Per Approved Procedure</t>
+  </si>
+  <si>
+    <t>Fire Alarm System Testing</t>
+  </si>
+  <si>
+    <t>Painting of Fire Fighting Pipe</t>
+  </si>
+  <si>
+    <t>Red / As Approved</t>
+  </si>
+  <si>
+    <t>Touch-up Painting</t>
+  </si>
+  <si>
+    <t>Fire Stopping / Sealing</t>
+  </si>
+  <si>
+    <t>Pipe/ Equipment Shifting</t>
+  </si>
+  <si>
+    <t>LOCATION</t>
   </si>
 </sst>
 </file>
@@ -162,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -175,6 +627,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -694,4 +1149,1189 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45289D9A-64B0-4FB7-A336-E82569DA4434}">
+  <dimension ref="A1:G56"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="6.6328125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="31.7265625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="37.7265625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6328125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="10.90625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7265625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="17.08984375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D16" s="2"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="2"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" s="2"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D27" s="2"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D29" s="2"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D42" s="2"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43" s="2">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D43" s="2"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D44" s="2"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D45" s="2"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="2">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D46" s="2"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="2">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D47" s="2"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" s="2">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D48" s="2"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="2">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D49" s="2"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D50" s="2"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D51" s="2"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="2">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D52" s="2"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="2">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D53" s="2"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54" s="2">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D54" s="2"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55" s="2">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D55" s="2"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56" s="2">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D56" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="63" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4AD9576-1618-48F3-9CB5-E51FE43263AE}">
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="19.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.26953125" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>